<commit_message>
Adding experiments from SPI
</commit_message>
<xml_diff>
--- a/Res_ConvLSTM/DroughtDataset_model_testing_1753444629_h_10.xlsx
+++ b/Res_ConvLSTM/DroughtDataset_model_testing_1753444629_h_10.xlsx
@@ -658,7 +658,7 @@
         <v>0.00845820783045732</v>
       </c>
       <c r="C2" t="n">
-        <v>63129780</v>
+        <v>6312978</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -679,49 +679,49 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>63129780</v>
+        <v>6312978</v>
       </c>
       <c r="K2" t="n">
-        <v>41582544</v>
+        <v>4172274</v>
       </c>
       <c r="L2" t="n">
-        <v>15564444</v>
+        <v>1533271</v>
       </c>
       <c r="M2" t="n">
-        <v>2882640</v>
+        <v>283962</v>
       </c>
       <c r="N2" t="n">
-        <v>64085</v>
+        <v>6572</v>
       </c>
       <c r="O2" t="n">
-        <v>1725018</v>
+        <v>170358</v>
       </c>
       <c r="P2" t="n">
-        <v>31776</v>
+        <v>3182</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.9999263882637024</v>
+        <v>0.9999447464942932</v>
       </c>
       <c r="R2" t="n">
-        <v>0.7133088707923889</v>
+        <v>0.7034690380096436</v>
       </c>
       <c r="S2" t="n">
-        <v>0.5367839336395264</v>
+        <v>0.5424830913543701</v>
       </c>
       <c r="T2" t="n">
-        <v>0.4040066599845886</v>
+        <v>0.4093181490898132</v>
       </c>
       <c r="U2" t="n">
-        <v>0.04559178650379181</v>
+        <v>0.04662580043077469</v>
       </c>
       <c r="V2" t="n">
-        <v>0.4049816131591797</v>
+        <v>0.408363938331604</v>
       </c>
       <c r="W2" t="n">
-        <v>0.4520121216773987</v>
+        <v>0.4537934958934784</v>
       </c>
       <c r="X2" t="n">
-        <v>63129780</v>
+        <v>6312978</v>
       </c>
       <c r="Y2" t="n">
         <v>0</v>
@@ -742,46 +742,46 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>63129780</v>
+        <v>6312978</v>
       </c>
       <c r="AF2" t="n">
-        <v>47949558</v>
+        <v>4750163</v>
       </c>
       <c r="AG2" t="n">
-        <v>29849211</v>
+        <v>3018205</v>
       </c>
       <c r="AH2" t="n">
-        <v>8017135</v>
+        <v>806591</v>
       </c>
       <c r="AI2" t="n">
-        <v>590732</v>
+        <v>59281</v>
       </c>
       <c r="AJ2" t="n">
-        <v>4597593</v>
+        <v>461241</v>
       </c>
       <c r="AK2" t="n">
-        <v>1801493</v>
+        <v>180417</v>
       </c>
       <c r="AL2" t="n">
         <v>1</v>
       </c>
       <c r="AM2" t="n">
-        <v>0.9559409618377686</v>
+        <v>0.9546809196472168</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.9116660952568054</v>
+        <v>0.9128581881523132</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.8582287430763245</v>
+        <v>0.8581860065460205</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.6617533564567566</v>
+        <v>0.6609027981758118</v>
       </c>
       <c r="AQ2" t="n">
-        <v>0.902009129524231</v>
+        <v>0.901951789855957</v>
       </c>
       <c r="AR2" t="n">
-        <v>0.9314513206481934</v>
+        <v>0.9314922094345093</v>
       </c>
     </row>
     <row r="3">
@@ -792,130 +792,130 @@
         <v>0.002027664927559576</v>
       </c>
       <c r="C3" t="n">
-        <v>612</v>
+        <v>70</v>
       </c>
       <c r="D3" t="n">
-        <v>41582544</v>
+        <v>4172274</v>
       </c>
       <c r="E3" t="n">
-        <v>8076976</v>
+        <v>750096</v>
       </c>
       <c r="F3" t="n">
-        <v>346057</v>
+        <v>31275</v>
       </c>
       <c r="G3" t="n">
-        <v>38505</v>
+        <v>3644</v>
       </c>
       <c r="H3" t="n">
-        <v>29695</v>
+        <v>2627</v>
       </c>
       <c r="I3" t="n">
-        <v>1351</v>
+        <v>126</v>
       </c>
       <c r="J3" t="n">
-        <v>100161571</v>
+        <v>10016273</v>
       </c>
       <c r="K3" t="n">
-        <v>96507518</v>
+        <v>9610763</v>
       </c>
       <c r="L3" t="n">
-        <v>117055391</v>
+        <v>11717345</v>
       </c>
       <c r="M3" t="n">
-        <v>149690957</v>
+        <v>14977962</v>
       </c>
       <c r="N3" t="n">
-        <v>161060895</v>
+        <v>16105412</v>
       </c>
       <c r="O3" t="n">
-        <v>155661091</v>
+        <v>15570877</v>
       </c>
       <c r="P3" t="n">
-        <v>161322864</v>
+        <v>16131965</v>
       </c>
       <c r="Q3" t="n">
         <v>1</v>
       </c>
       <c r="R3" t="n">
-        <v>0.8303930163383484</v>
+        <v>0.84116530418396</v>
       </c>
       <c r="S3" t="n">
-        <v>0.4743909239768982</v>
+        <v>0.4619493782520294</v>
       </c>
       <c r="T3" t="n">
-        <v>0.3082195818424225</v>
+        <v>0.3014919459819794</v>
       </c>
       <c r="U3" t="n">
-        <v>0.07171842455863953</v>
+        <v>0.07317833602428436</v>
       </c>
       <c r="V3" t="n">
-        <v>0.3382103145122528</v>
+        <v>0.3327896296977997</v>
       </c>
       <c r="W3" t="n">
-        <v>0.0164249911904335</v>
+        <v>0.01641856506466866</v>
       </c>
       <c r="X3" t="n">
         <v>0</v>
       </c>
       <c r="Y3" t="n">
-        <v>47949558</v>
+        <v>4750163</v>
       </c>
       <c r="Z3" t="n">
-        <v>1972670</v>
+        <v>194702</v>
       </c>
       <c r="AA3" t="n">
-        <v>84826</v>
+        <v>8398</v>
       </c>
       <c r="AB3" t="n">
-        <v>68106</v>
+        <v>6808</v>
       </c>
       <c r="AC3" t="n">
-        <v>280</v>
+        <v>11</v>
       </c>
       <c r="AD3" t="n">
-        <v>300</v>
+        <v>30</v>
       </c>
       <c r="AE3" t="n">
-        <v>100166220</v>
+        <v>10016622</v>
       </c>
       <c r="AF3" t="n">
-        <v>111010280</v>
+        <v>11143996</v>
       </c>
       <c r="AG3" t="n">
-        <v>127594505</v>
+        <v>12722349</v>
       </c>
       <c r="AH3" t="n">
-        <v>152619092</v>
+        <v>15254456</v>
       </c>
       <c r="AI3" t="n">
-        <v>162100491</v>
+        <v>16209376</v>
       </c>
       <c r="AJ3" t="n">
-        <v>157696105</v>
+        <v>15767551</v>
       </c>
       <c r="AK3" t="n">
-        <v>161228809</v>
+        <v>16122526</v>
       </c>
       <c r="AL3" t="n">
         <v>1</v>
       </c>
       <c r="AM3" t="n">
-        <v>0.9575406908988953</v>
+        <v>0.9576725363731384</v>
       </c>
       <c r="AN3" t="n">
-        <v>0.9097784161567688</v>
+        <v>0.9093356132507324</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.85721355676651</v>
+        <v>0.8563846349716187</v>
       </c>
       <c r="AP3" t="n">
-        <v>0.661096453666687</v>
+        <v>0.6600859761238098</v>
       </c>
       <c r="AQ3" t="n">
-        <v>0.9014128446578979</v>
+        <v>0.9010214805603027</v>
       </c>
       <c r="AR3" t="n">
-        <v>0.9311903715133667</v>
+        <v>0.9309202432632446</v>
       </c>
     </row>
     <row r="4">
@@ -926,285 +926,285 @@
         <v>0.03198836053224347</v>
       </c>
       <c r="C4" t="n">
-        <v>295</v>
+        <v>41</v>
       </c>
       <c r="D4" t="n">
-        <v>14833297</v>
+        <v>1557043</v>
       </c>
       <c r="E4" t="n">
-        <v>15564444</v>
+        <v>1533271</v>
       </c>
       <c r="F4" t="n">
-        <v>1878356</v>
+        <v>177331</v>
       </c>
       <c r="G4" t="n">
-        <v>213503</v>
+        <v>21011</v>
       </c>
       <c r="H4" t="n">
-        <v>314131</v>
+        <v>29931</v>
       </c>
       <c r="I4" t="n">
-        <v>5294</v>
+        <v>504</v>
       </c>
       <c r="J4" t="n">
-        <v>4649</v>
+        <v>349</v>
       </c>
       <c r="K4" t="n">
-        <v>16712742</v>
+        <v>1758725</v>
       </c>
       <c r="L4" t="n">
-        <v>13431289</v>
+        <v>1293123</v>
       </c>
       <c r="M4" t="n">
-        <v>4252490</v>
+        <v>409782</v>
       </c>
       <c r="N4" t="n">
-        <v>1341541</v>
+        <v>134380</v>
       </c>
       <c r="O4" t="n">
-        <v>2534479</v>
+        <v>246814</v>
       </c>
       <c r="P4" t="n">
-        <v>38523</v>
+        <v>3830</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.9999632239341736</v>
+        <v>0.999972403049469</v>
       </c>
       <c r="R4" t="n">
-        <v>0.7674107551574707</v>
+        <v>0.7661797404289246</v>
       </c>
       <c r="S4" t="n">
-        <v>0.5036624670028687</v>
+        <v>0.4989877045154572</v>
       </c>
       <c r="T4" t="n">
-        <v>0.3496719002723694</v>
+        <v>0.3472267389297485</v>
       </c>
       <c r="U4" t="n">
-        <v>0.05574572086334229</v>
+        <v>0.0569596104323864</v>
       </c>
       <c r="V4" t="n">
-        <v>0.3685964345932007</v>
+        <v>0.3667236864566803</v>
       </c>
       <c r="W4" t="n">
-        <v>0.03169815242290497</v>
+        <v>0.03169054165482521</v>
       </c>
       <c r="X4" t="n">
         <v>0</v>
       </c>
       <c r="Y4" t="n">
-        <v>2063963</v>
+        <v>210743</v>
       </c>
       <c r="Z4" t="n">
-        <v>29849211</v>
+        <v>3018205</v>
       </c>
       <c r="AA4" t="n">
-        <v>828823</v>
+        <v>83377</v>
       </c>
       <c r="AB4" t="n">
-        <v>55262</v>
+        <v>5608</v>
       </c>
       <c r="AC4" t="n">
-        <v>11381</v>
+        <v>1131</v>
       </c>
       <c r="AD4" t="n">
-        <v>680</v>
+        <v>68</v>
       </c>
       <c r="AE4" t="n">
         <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>2209980</v>
+        <v>225492</v>
       </c>
       <c r="AG4" t="n">
-        <v>2892175</v>
+        <v>288119</v>
       </c>
       <c r="AH4" t="n">
-        <v>1324355</v>
+        <v>133288</v>
       </c>
       <c r="AI4" t="n">
-        <v>301945</v>
+        <v>30416</v>
       </c>
       <c r="AJ4" t="n">
-        <v>499465</v>
+        <v>50140</v>
       </c>
       <c r="AK4" t="n">
-        <v>132578</v>
+        <v>13269</v>
       </c>
       <c r="AL4" t="n">
         <v>1</v>
       </c>
       <c r="AM4" t="n">
-        <v>0.9567400813102722</v>
+        <v>0.956174373626709</v>
       </c>
       <c r="AN4" t="n">
-        <v>0.9107212424278259</v>
+        <v>0.9110934734344482</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.8577207922935486</v>
+        <v>0.8572843670845032</v>
       </c>
       <c r="AP4" t="n">
-        <v>0.6614247560501099</v>
+        <v>0.6604941487312317</v>
       </c>
       <c r="AQ4" t="n">
-        <v>0.9017109274864197</v>
+        <v>0.9014863967895508</v>
       </c>
       <c r="AR4" t="n">
-        <v>0.93132084608078</v>
+        <v>0.9312061071395874</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="n">
-        <v>627</v>
+        <v>51</v>
       </c>
       <c r="D5" t="n">
-        <v>1391025</v>
+        <v>149374</v>
       </c>
       <c r="E5" t="n">
-        <v>3954083</v>
+        <v>398431</v>
       </c>
       <c r="F5" t="n">
-        <v>2882640</v>
+        <v>283962</v>
       </c>
       <c r="G5" t="n">
-        <v>348295</v>
+        <v>34956</v>
       </c>
       <c r="H5" t="n">
-        <v>766411</v>
+        <v>74081</v>
       </c>
       <c r="I5" t="n">
-        <v>9472</v>
+        <v>1001</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>8493196</v>
+        <v>787838</v>
       </c>
       <c r="L5" t="n">
-        <v>17244876</v>
+        <v>1785861</v>
       </c>
       <c r="M5" t="n">
-        <v>6469913</v>
+        <v>657894</v>
       </c>
       <c r="N5" t="n">
-        <v>829479</v>
+        <v>83236</v>
       </c>
       <c r="O5" t="n">
-        <v>3375412</v>
+        <v>341551</v>
       </c>
       <c r="P5" t="n">
-        <v>1902837</v>
+        <v>190623</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.9999715089797974</v>
+        <v>0.9999786019325256</v>
       </c>
       <c r="R5" t="n">
-        <v>0.845642626285553</v>
+        <v>0.8440523147583008</v>
       </c>
       <c r="S5" t="n">
-        <v>0.8121438026428223</v>
+        <v>0.8114476799964905</v>
       </c>
       <c r="T5" t="n">
-        <v>0.9343376159667969</v>
+        <v>0.9346171617507935</v>
       </c>
       <c r="U5" t="n">
-        <v>0.9867050051689148</v>
+        <v>0.9866735339164734</v>
       </c>
       <c r="V5" t="n">
-        <v>0.9638087153434753</v>
+        <v>0.9639694094657898</v>
       </c>
       <c r="W5" t="n">
-        <v>0.9881113767623901</v>
+        <v>0.9880920052528381</v>
       </c>
       <c r="X5" t="n">
         <v>0</v>
       </c>
       <c r="Y5" t="n">
-        <v>80454</v>
+        <v>8120</v>
       </c>
       <c r="Z5" t="n">
-        <v>857060</v>
+        <v>87176</v>
       </c>
       <c r="AA5" t="n">
-        <v>8017135</v>
+        <v>806591</v>
       </c>
       <c r="AB5" t="n">
-        <v>99758</v>
+        <v>10039</v>
       </c>
       <c r="AC5" t="n">
-        <v>291816</v>
+        <v>29297</v>
       </c>
       <c r="AD5" t="n">
-        <v>6330</v>
+        <v>633</v>
       </c>
       <c r="AE5" t="n">
         <v>0</v>
       </c>
       <c r="AF5" t="n">
-        <v>2126182</v>
+        <v>209949</v>
       </c>
       <c r="AG5" t="n">
-        <v>2960109</v>
+        <v>300927</v>
       </c>
       <c r="AH5" t="n">
-        <v>1335418</v>
+        <v>135265</v>
       </c>
       <c r="AI5" t="n">
-        <v>302832</v>
+        <v>30527</v>
       </c>
       <c r="AJ5" t="n">
-        <v>502837</v>
+        <v>50668</v>
       </c>
       <c r="AK5" t="n">
-        <v>133120</v>
+        <v>13388</v>
       </c>
       <c r="AL5" t="n">
         <v>1</v>
       </c>
       <c r="AM5" t="n">
-        <v>0.9734460115432739</v>
+        <v>0.9733342528343201</v>
       </c>
       <c r="AN5" t="n">
-        <v>0.9641615152359009</v>
+        <v>0.963927686214447</v>
       </c>
       <c r="AO5" t="n">
-        <v>0.9837119579315186</v>
+        <v>0.9835542440414429</v>
       </c>
       <c r="AP5" t="n">
-        <v>0.9962964653968811</v>
+        <v>0.9962679147720337</v>
       </c>
       <c r="AQ5" t="n">
-        <v>0.9938620328903198</v>
+        <v>0.993826687335968</v>
       </c>
       <c r="AR5" t="n">
-        <v>0.9983729124069214</v>
+        <v>0.9983675479888916</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
-        <v>361</v>
+        <v>20</v>
       </c>
       <c r="D6" t="n">
-        <v>248619</v>
+        <v>26509</v>
       </c>
       <c r="E6" t="n">
-        <v>259808</v>
+        <v>25765</v>
       </c>
       <c r="F6" t="n">
-        <v>237992</v>
+        <v>23007</v>
       </c>
       <c r="G6" t="n">
-        <v>64085</v>
+        <v>6572</v>
       </c>
       <c r="H6" t="n">
-        <v>80575</v>
+        <v>7765</v>
       </c>
       <c r="I6" t="n">
-        <v>2124</v>
+        <v>170</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -1224,22 +1224,22 @@
         <v>0</v>
       </c>
       <c r="Y6" t="n">
-        <v>65084</v>
+        <v>6593</v>
       </c>
       <c r="Z6" t="n">
-        <v>53535</v>
+        <v>5350</v>
       </c>
       <c r="AA6" t="n">
-        <v>109471</v>
+        <v>11081</v>
       </c>
       <c r="AB6" t="n">
-        <v>590732</v>
+        <v>59281</v>
       </c>
       <c r="AC6" t="n">
-        <v>69932</v>
+        <v>7022</v>
       </c>
       <c r="AD6" t="n">
-        <v>4810</v>
+        <v>481</v>
       </c>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr"/>
@@ -1260,25 +1260,25 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="n">
-        <v>1223</v>
+        <v>59</v>
       </c>
       <c r="D7" t="n">
-        <v>218641</v>
+        <v>23363</v>
       </c>
       <c r="E7" t="n">
-        <v>1012460</v>
+        <v>105225</v>
       </c>
       <c r="F7" t="n">
-        <v>1528142</v>
+        <v>151722</v>
       </c>
       <c r="G7" t="n">
-        <v>594664</v>
+        <v>59153</v>
       </c>
       <c r="H7" t="n">
-        <v>1725018</v>
+        <v>170358</v>
       </c>
       <c r="I7" t="n">
-        <v>20282</v>
+        <v>2029</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -1298,22 +1298,22 @@
         <v>0</v>
       </c>
       <c r="Y7" t="n">
-        <v>199</v>
+        <v>8</v>
       </c>
       <c r="Z7" t="n">
-        <v>8100</v>
+        <v>810</v>
       </c>
       <c r="AA7" t="n">
-        <v>297921</v>
+        <v>30099</v>
       </c>
       <c r="AB7" t="n">
-        <v>76159</v>
+        <v>7694</v>
       </c>
       <c r="AC7" t="n">
-        <v>4597593</v>
+        <v>461241</v>
       </c>
       <c r="AD7" t="n">
-        <v>120458</v>
+        <v>12057</v>
       </c>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
@@ -1334,25 +1334,25 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>1531</v>
+        <v>108</v>
       </c>
       <c r="D8" t="n">
-        <v>21160</v>
+        <v>2436</v>
       </c>
       <c r="E8" t="n">
-        <v>127962</v>
+        <v>13606</v>
       </c>
       <c r="F8" t="n">
-        <v>261943</v>
+        <v>26447</v>
       </c>
       <c r="G8" t="n">
-        <v>146574</v>
+        <v>15616</v>
       </c>
       <c r="H8" t="n">
-        <v>1343667</v>
+        <v>132410</v>
       </c>
       <c r="I8" t="n">
-        <v>31776</v>
+        <v>3182</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -1372,22 +1372,22 @@
         <v>0</v>
       </c>
       <c r="Y8" t="n">
-        <v>280</v>
+        <v>28</v>
       </c>
       <c r="Z8" t="n">
-        <v>810</v>
+        <v>81</v>
       </c>
       <c r="AA8" t="n">
-        <v>3314</v>
+        <v>333</v>
       </c>
       <c r="AB8" t="n">
-        <v>2660</v>
+        <v>267</v>
       </c>
       <c r="AC8" t="n">
-        <v>126056</v>
+        <v>12679</v>
       </c>
       <c r="AD8" t="n">
-        <v>1801493</v>
+        <v>180417</v>
       </c>
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr"/>

</xml_diff>